<commit_message>
📊 [auto] Economic data update — 2026-10-27 18:30 UTC
</commit_message>
<xml_diff>
--- a/reports/excel/MacroPulse_2026-10-27.xlsx
+++ b/reports/excel/MacroPulse_2026-10-27.xlsx
@@ -651,7 +651,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-10-27 01:34 UTC</t>
+          <t>MacroPulse 總體經濟指標報告　　生成時間：2026-10-27 18:30 UTC</t>
         </is>
       </c>
     </row>
@@ -1360,12 +1360,12 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>3.386e+05</t>
+          <t>3.454e+05</t>
         </is>
       </c>
       <c r="G13" s="4" t="inlineStr">
@@ -1375,7 +1375,7 @@
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>9.94%</t>
         </is>
       </c>
       <c r="I13" s="4" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>1.84%</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
@@ -2724,12 +2724,12 @@
       </c>
       <c r="E35" s="5" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>684</t>
+          <t>676</t>
         </is>
       </c>
       <c r="G35" s="4" t="inlineStr">
@@ -2739,7 +2739,7 @@
       </c>
       <c r="H35" s="5" t="inlineStr">
         <is>
-          <t>-2.01%</t>
+          <t>-5.32%</t>
         </is>
       </c>
       <c r="I35" s="4" t="inlineStr">
@@ -2749,7 +2749,7 @@
       </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>6.38%</t>
+          <t>-0.59%</t>
         </is>
       </c>
       <c r="K35" s="4" t="inlineStr">
@@ -2866,7 +2866,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🔥 通膨指標　歷史數據　　生成時間：2026-10-27 01:34 UTC</t>
+          <t>🔥 通膨指標　歷史數據　　生成時間：2026-10-27 18:30 UTC</t>
         </is>
       </c>
     </row>
@@ -14688,7 +14688,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>📈 經濟成長　歷史數據　　生成時間：2026-10-27 01:34 UTC</t>
+          <t>📈 經濟成長　歷史數據　　生成時間：2026-10-27 18:30 UTC</t>
         </is>
       </c>
     </row>
@@ -24473,12 +24473,12 @@
       </c>
       <c r="O121" s="20" t="inlineStr">
         <is>
-          <t>11.76%</t>
+          <t>11.77%</t>
         </is>
       </c>
       <c r="P121" s="20" t="inlineStr">
         <is>
-          <t>0.86%</t>
+          <t>0.87%</t>
         </is>
       </c>
     </row>
@@ -24550,17 +24550,17 @@
       </c>
       <c r="N122" s="19" t="inlineStr">
         <is>
-          <t>3.386e+05</t>
+          <t>3.391e+05</t>
         </is>
       </c>
       <c r="O122" s="19" t="inlineStr">
         <is>
-          <t>8.48%</t>
+          <t>8.64%</t>
         </is>
       </c>
       <c r="P122" s="19" t="inlineStr">
         <is>
-          <t>-0.02%</t>
+          <t>0.12%</t>
         </is>
       </c>
     </row>
@@ -24632,17 +24632,17 @@
       </c>
       <c r="N123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>3.454e+05</t>
         </is>
       </c>
       <c r="O123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>9.94%</t>
         </is>
       </c>
       <c r="P123" s="20" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>1.84%</t>
         </is>
       </c>
     </row>
@@ -24692,7 +24692,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>👷 勞動市場　歷史數據　　生成時間：2026-10-27 01:34 UTC</t>
+          <t>👷 勞動市場　歷史數據　　生成時間：2026-10-27 18:30 UTC</t>
         </is>
       </c>
     </row>
@@ -36517,7 +36517,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏦 利率與債券　歷史數據　　生成時間：2026-10-27 01:34 UTC</t>
+          <t>🏦 利率與債券　歷史數據　　生成時間：2026-10-27 18:30 UTC</t>
         </is>
       </c>
     </row>
@@ -48336,7 +48336,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>💭 信心指數　歷史數據　　生成時間：2026-10-27 01:34 UTC</t>
+          <t>💭 信心指數　歷史數據　　生成時間：2026-10-27 18:30 UTC</t>
         </is>
       </c>
     </row>
@@ -56513,7 +56513,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-10-27 01:34 UTC</t>
+          <t>⚠️ 信用與違約　歷史數據　　生成時間：2026-10-27 18:30 UTC</t>
         </is>
       </c>
     </row>
@@ -59729,7 +59729,7 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>🏠 房市　歷史數據　　生成時間：2026-10-27 01:34 UTC</t>
+          <t>🏠 房市　歷史數據　　生成時間：2026-10-27 18:30 UTC</t>
         </is>
       </c>
     </row>
@@ -59830,7 +59830,7 @@
       </c>
       <c r="E4" s="19" t="inlineStr">
         <is>
-          <t>733</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="F4" s="19" t="inlineStr">
@@ -59892,7 +59892,7 @@
       </c>
       <c r="G5" s="20" t="inlineStr">
         <is>
-          <t>-6.00%</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="H5" s="20" t="inlineStr">
@@ -60459,7 +60459,7 @@
       </c>
       <c r="F16" s="19" t="inlineStr">
         <is>
-          <t>-24.69%</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G16" s="19" t="inlineStr">
@@ -62794,17 +62794,17 @@
       </c>
       <c r="E61" s="20" t="inlineStr">
         <is>
-          <t>672</t>
+          <t>680</t>
         </is>
       </c>
       <c r="F61" s="20" t="inlineStr">
         <is>
-          <t>1.05%</t>
+          <t>2.26%</t>
         </is>
       </c>
       <c r="G61" s="20" t="inlineStr">
         <is>
-          <t>5.66%</t>
+          <t>6.92%</t>
         </is>
       </c>
       <c r="H61" s="20" t="inlineStr">
@@ -62846,17 +62846,17 @@
       </c>
       <c r="E62" s="19" t="inlineStr">
         <is>
-          <t>643</t>
+          <t>647</t>
         </is>
       </c>
       <c r="F62" s="19" t="inlineStr">
         <is>
-          <t>-0.77%</t>
+          <t>-0.15%</t>
         </is>
       </c>
       <c r="G62" s="19" t="inlineStr">
         <is>
-          <t>-4.32%</t>
+          <t>-4.85%</t>
         </is>
       </c>
       <c r="H62" s="19" t="inlineStr">
@@ -62898,17 +62898,17 @@
       </c>
       <c r="E63" s="20" t="inlineStr">
         <is>
-          <t>684</t>
+          <t>680</t>
         </is>
       </c>
       <c r="F63" s="20" t="inlineStr">
         <is>
-          <t>-2.01%</t>
+          <t>-2.58%</t>
         </is>
       </c>
       <c r="G63" s="20" t="inlineStr">
         <is>
-          <t>6.38%</t>
+          <t>5.10%</t>
         </is>
       </c>
       <c r="H63" s="20" t="inlineStr">
@@ -62950,17 +62950,17 @@
       </c>
       <c r="E64" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>676</t>
         </is>
       </c>
       <c r="F64" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-5.32%</t>
         </is>
       </c>
       <c r="G64" s="19" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>-0.59%</t>
         </is>
       </c>
       <c r="H64" s="19" t="inlineStr">

</xml_diff>